<commit_message>
feat: add scrapers for multiple banks, implement bulk bank update utility, and deploy API integration
</commit_message>
<xml_diff>
--- a/input/banks.xlsx
+++ b/input/banks.xlsx
@@ -1,44 +1,199 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Blostem-projects\web scrape\input\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA2798E4-DDB3-4994-804F-E52B35AB51CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Banks" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+  <si>
+    <t>Bank Name</t>
+  </si>
+  <si>
+    <t>FD URL</t>
+  </si>
+  <si>
+    <t>HDFC Bank</t>
+  </si>
+  <si>
+    <t>https://www.hdfcbank.com/personal/save/deposits/fixed-deposit-interest-rates</t>
+  </si>
+  <si>
+    <t>SBI</t>
+  </si>
+  <si>
+    <t>https://sbi.co.in/web/interest-rates/deposit-rates/retail-domestic-term-deposits</t>
+  </si>
+  <si>
+    <t>ICICI Bank</t>
+  </si>
+  <si>
+    <t>https://www.icicibank.com/personal-banking/deposits/fixed-deposit/fd-interest-rates</t>
+  </si>
+  <si>
+    <t>Axis Bank</t>
+  </si>
+  <si>
+    <t>https://www.axis.bank.in/docs/default-source/default-document-library/interest-rates/domestic-fixed-deposits-06-june-26.pdf?sfvrsn=5eb4a7d0_1</t>
+  </si>
+  <si>
+    <t>Kotak Mahindra Bank</t>
+  </si>
+  <si>
+    <t>https://www.kotak.com/en/rates/interest-rates.html</t>
+  </si>
+  <si>
+    <t>PNB</t>
+  </si>
+  <si>
+    <t>https://www.pnbindia.in/interest-rates-deposit.html</t>
+  </si>
+  <si>
+    <t>IndusInd Bank</t>
+  </si>
+  <si>
+    <t>https://www.indusind.bank.in/in/en/personal/rates.html</t>
+  </si>
+  <si>
+    <t>Yes Bank</t>
+  </si>
+  <si>
+    <t>https://www.yes.bank.in/personal-banking/yes-individual/deposits/fixed-deposit</t>
+  </si>
+  <si>
+    <t>IDFC First Bank</t>
+  </si>
+  <si>
+    <t>https://www.idfcfirstbank.com/personal-banking/deposits/fixed-deposit/fd-interest-rates</t>
+  </si>
+  <si>
+    <t>Indian Overseas Bank</t>
+  </si>
+  <si>
+    <t>https://www.iob.bank.in/en/domestic-nro-nre-retail-term-deposit-rates</t>
+  </si>
+  <si>
+    <t>South Indian Bank</t>
+  </si>
+  <si>
+    <t>https://www.southindianbank.com/interestrates/interestrates.aspx</t>
+  </si>
+  <si>
+    <t>Federal Bank</t>
+  </si>
+  <si>
+    <t>https://www.federalbank.co.in/interest-rates</t>
+  </si>
+  <si>
+    <t>Canara Bank</t>
+  </si>
+  <si>
+    <t>https://www.canarabank.bank.in/pages/deposit-interest-rates</t>
+  </si>
+  <si>
+    <t>Bank of Baroda</t>
+  </si>
+  <si>
+    <t>https://www.bankbazaar.com/fixed-deposit/bank-of-baroda-fixed-deposit-rate.html</t>
+  </si>
+  <si>
+    <t>Bank of India</t>
+  </si>
+  <si>
+    <t>https://www.bankbazaar.com/fixed-deposit/bank-of-india-fixed-deposit-rate.html</t>
+  </si>
+  <si>
+    <t>Bank of Maharashtra</t>
+  </si>
+  <si>
+    <t>https://www.bankbazaar.com/fixed-deposit/bank-of-maharashtra-fixed-deposit-rate.html</t>
+  </si>
+  <si>
+    <t>RBL Bank</t>
+  </si>
+  <si>
+    <t>https://www.bankbazaar.com/fixed-deposit/rbl-bank-fixed-deposit-rate.html</t>
+  </si>
+  <si>
+    <t>IDBI Bank</t>
+  </si>
+  <si>
+    <t>https://www.bankbazaar.com/fixed-deposit/idbi-fixed-deposit-rate.html</t>
+  </si>
+  <si>
+    <t>Indian Bank</t>
+  </si>
+  <si>
+    <t>https://www.bankbazaar.com/fixed-deposit/indian-bank-fixed-deposit-rate.html</t>
+  </si>
+  <si>
+    <t>Central Bank of India</t>
+  </si>
+  <si>
+    <t>https://www.bankbazaar.com/fixed-deposit/central-bank-of-india-fixed-deposit-rate.html</t>
+  </si>
+  <si>
+    <t>Bandhan Bank</t>
+  </si>
+  <si>
+    <t>https://www.bankbazaar.com/fixed-deposit/bandhan-bank-fixed-deposit-rate.html</t>
+  </si>
+  <si>
+    <t>PNB Housing Finance</t>
+  </si>
+  <si>
+    <t>https://www.bankbazaar.com/fixed-deposit/pnbhfl-fixed-deposit-rate.html</t>
+  </si>
+  <si>
+    <t>KTDFC</t>
+  </si>
+  <si>
+    <t>https://www.bankbazaar.com/fixed-deposit/ktdfc-fixed-deposit-rate.html</t>
+  </si>
+  <si>
+    <t>LIC Housing Finance</t>
+  </si>
+  <si>
+    <t>https://www.bankbazaar.com/fixed-deposit/lic-housing-fixed-deposit-rate.html</t>
+  </si>
+  <si>
+    <t>Shriram Finance</t>
+  </si>
+  <si>
+    <t>https://www.bankbazaar.com/fixed-deposit/shriram-finance-fixed-deposit-rate.html</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -61,17 +216,28 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,116 +562,225 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Bank Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>FD URL</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>HDFC Bank</v>
-      </c>
-      <c r="B2" t="str">
-        <v>https://www.hdfcbank.com/personal/save/deposits/fixed-deposit-interest-rates</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>SBI</v>
-      </c>
-      <c r="B3" t="str">
-        <v>https://sbi.co.in/web/interest-rates/deposit-rates/retail-domestic-term-deposits</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>ICICI Bank</v>
-      </c>
-      <c r="B4" t="str">
-        <v>https://www.icicibank.com/personal-banking/deposits/fixed-deposit/fd-interest-rates</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Axis Bank</v>
-      </c>
-      <c r="B5" t="str">
-        <v>https://www.axis.bank.in/docs/default-source/default-document-library/interest-rates/domestic-fixed-deposits-06-june-26.pdf?sfvrsn=5eb4a7d0_1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Kotak Mahindra Bank</v>
-      </c>
-      <c r="B6" t="str">
-        <v>https://www.kotak.com/en/rates/interest-rates.html</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>PNB</v>
-      </c>
-      <c r="B7" t="str">
-        <v>https://www.pnbindia.in/interest-rates-deposit.html</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>IndusInd Bank</v>
-      </c>
-      <c r="B8" t="str">
-        <v>https://www.indusind.bank.in/in/en/personal/rates.html</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Yes Bank</v>
-      </c>
-      <c r="B9" t="str">
-        <v>https://www.yes.bank.in/personal-banking/yes-individual/deposits/fixed-deposit</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>IDFC First Bank</v>
-      </c>
-      <c r="B10" t="str">
-        <v>https://www.idfcfirstbank.com/personal-banking/deposits/fixed-deposit/fd-interest-rates</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Indian Overseas Bank</v>
-      </c>
-      <c r="B11" t="str">
-        <v>https://www.iob.bank.in/en/domestic-nro-nre-retail-term-deposit-rates</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>South Indian Bank</v>
-      </c>
-      <c r="B12" t="str">
-        <v>https://www.southindianbank.com/interestrates/interestrates.aspx</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Federal Bank</v>
-      </c>
-      <c r="B13" t="str">
-        <v>https://www.federalbank.co.in/interest-rates</v>
+    <row r="1" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{14821128-51C9-413E-908B-AF4C53380BDE}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
+    <ignoredError sqref="A1:B4 A6:B26 A5" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>